<commit_message>
Keep only the word-to-meaning questions
Drops the second round, which asked the question backwards ("Which word
means ...?"), leaving ten questions that each show a word and ask what it
means. The retired round took the round chip, the per-question kicker
switch and the "missed both ways" tally with it, since a word is now asked
exactly once.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013RMGHQ6jfMwb6DtLJUeR7A
</commit_message>
<xml_diff>
--- a/kahoot/Kahoot-Vocab-Quiz-Import.xlsx
+++ b/kahoot/Kahoot-Vocab-Quiz-Import.xlsx
@@ -53,7 +53,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
@@ -63,11 +63,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="0046178F"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00F2EDFB"/>
       </patternFill>
     </fill>
   </fills>
@@ -83,7 +78,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -98,12 +93,6 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -472,7 +461,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G30"/>
+  <dimension ref="A1:G20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
@@ -896,340 +885,10 @@
         <v>2</v>
       </c>
     </row>
-    <row r="19" ht="30" customHeight="1">
-      <c r="A19" s="6" t="inlineStr">
-        <is>
-          <t>Which word means "hold back"?</t>
-        </is>
-      </c>
-      <c r="B19" s="6" t="inlineStr">
-        <is>
-          <t>accede</t>
-        </is>
-      </c>
-      <c r="C19" s="6" t="inlineStr">
-        <is>
-          <t>curtail</t>
-        </is>
-      </c>
-      <c r="D19" s="6" t="inlineStr">
-        <is>
-          <t>abstain</t>
-        </is>
-      </c>
-      <c r="E19" s="6" t="inlineStr">
-        <is>
-          <t>animate</t>
-        </is>
-      </c>
-      <c r="F19" s="7" t="n">
-        <v>20</v>
-      </c>
-      <c r="G19" s="7" t="n">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="20" ht="30" customHeight="1">
+    <row r="20">
       <c r="A20" s="6" t="inlineStr">
         <is>
-          <t>Which word means "to agree to a request or demand"?</t>
-        </is>
-      </c>
-      <c r="B20" s="6" t="inlineStr">
-        <is>
-          <t>accede</t>
-        </is>
-      </c>
-      <c r="C20" s="6" t="inlineStr">
-        <is>
-          <t>abstain</t>
-        </is>
-      </c>
-      <c r="D20" s="6" t="inlineStr">
-        <is>
-          <t>accessible</t>
-        </is>
-      </c>
-      <c r="E20" s="6" t="inlineStr">
-        <is>
-          <t>cordial</t>
-        </is>
-      </c>
-      <c r="F20" s="7" t="n">
-        <v>20</v>
-      </c>
-      <c r="G20" s="7" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="21" ht="30" customHeight="1">
-      <c r="A21" s="6" t="inlineStr">
-        <is>
-          <t>Which word means "obtainable"?</t>
-        </is>
-      </c>
-      <c r="B21" s="6" t="inlineStr">
-        <is>
-          <t>affluent</t>
-        </is>
-      </c>
-      <c r="C21" s="6" t="inlineStr">
-        <is>
-          <t>accede</t>
-        </is>
-      </c>
-      <c r="D21" s="6" t="inlineStr">
-        <is>
-          <t>diligent</t>
-        </is>
-      </c>
-      <c r="E21" s="6" t="inlineStr">
-        <is>
-          <t>accessible</t>
-        </is>
-      </c>
-      <c r="F21" s="7" t="n">
-        <v>20</v>
-      </c>
-      <c r="G21" s="7" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="22" ht="30" customHeight="1">
-      <c r="A22" s="6" t="inlineStr">
-        <is>
-          <t>Which word means "having a large amount of money or wealth"?</t>
-        </is>
-      </c>
-      <c r="B22" s="6" t="inlineStr">
-        <is>
-          <t>accessible</t>
-        </is>
-      </c>
-      <c r="C22" s="6" t="inlineStr">
-        <is>
-          <t>affluent</t>
-        </is>
-      </c>
-      <c r="D22" s="6" t="inlineStr">
-        <is>
-          <t>boisterous</t>
-        </is>
-      </c>
-      <c r="E22" s="6" t="inlineStr">
-        <is>
-          <t>cordial</t>
-        </is>
-      </c>
-      <c r="F22" s="7" t="n">
-        <v>20</v>
-      </c>
-      <c r="G22" s="7" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="23" ht="30" customHeight="1">
-      <c r="A23" s="6" t="inlineStr">
-        <is>
-          <t>Which word means "to make something alive; give it energy and spirit"?</t>
-        </is>
-      </c>
-      <c r="B23" s="6" t="inlineStr">
-        <is>
-          <t>animate</t>
-        </is>
-      </c>
-      <c r="C23" s="6" t="inlineStr">
-        <is>
-          <t>abstain</t>
-        </is>
-      </c>
-      <c r="D23" s="6" t="inlineStr">
-        <is>
-          <t>cunning</t>
-        </is>
-      </c>
-      <c r="E23" s="6" t="inlineStr">
-        <is>
-          <t>curtail</t>
-        </is>
-      </c>
-      <c r="F23" s="7" t="n">
-        <v>20</v>
-      </c>
-      <c r="G23" s="7" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="24" ht="30" customHeight="1">
-      <c r="A24" s="6" t="inlineStr">
-        <is>
-          <t>Which word means "loud, energetic"?</t>
-        </is>
-      </c>
-      <c r="B24" s="6" t="inlineStr">
-        <is>
-          <t>cordial</t>
-        </is>
-      </c>
-      <c r="C24" s="6" t="inlineStr">
-        <is>
-          <t>diligent</t>
-        </is>
-      </c>
-      <c r="D24" s="6" t="inlineStr">
-        <is>
-          <t>boisterous</t>
-        </is>
-      </c>
-      <c r="E24" s="6" t="inlineStr">
-        <is>
-          <t>affluent</t>
-        </is>
-      </c>
-      <c r="F24" s="7" t="n">
-        <v>20</v>
-      </c>
-      <c r="G24" s="7" t="n">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="25" ht="30" customHeight="1">
-      <c r="A25" s="6" t="inlineStr">
-        <is>
-          <t>Which word means "affectionate, politely warm"?</t>
-        </is>
-      </c>
-      <c r="B25" s="6" t="inlineStr">
-        <is>
-          <t>cunning</t>
-        </is>
-      </c>
-      <c r="C25" s="6" t="inlineStr">
-        <is>
-          <t>cordial</t>
-        </is>
-      </c>
-      <c r="D25" s="6" t="inlineStr">
-        <is>
-          <t>boisterous</t>
-        </is>
-      </c>
-      <c r="E25" s="6" t="inlineStr">
-        <is>
-          <t>accessible</t>
-        </is>
-      </c>
-      <c r="F25" s="7" t="n">
-        <v>20</v>
-      </c>
-      <c r="G25" s="7" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="26" ht="30" customHeight="1">
-      <c r="A26" s="6" t="inlineStr">
-        <is>
-          <t>Which word means "clever at being deceitful"?</t>
-        </is>
-      </c>
-      <c r="B26" s="6" t="inlineStr">
-        <is>
-          <t>cordial</t>
-        </is>
-      </c>
-      <c r="C26" s="6" t="inlineStr">
-        <is>
-          <t>diligent</t>
-        </is>
-      </c>
-      <c r="D26" s="6" t="inlineStr">
-        <is>
-          <t>animate</t>
-        </is>
-      </c>
-      <c r="E26" s="6" t="inlineStr">
-        <is>
-          <t>cunning</t>
-        </is>
-      </c>
-      <c r="F26" s="7" t="n">
-        <v>20</v>
-      </c>
-      <c r="G26" s="7" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="27" ht="30" customHeight="1">
-      <c r="A27" s="6" t="inlineStr">
-        <is>
-          <t>Which word means "reduce, restrict, shorten"?</t>
-        </is>
-      </c>
-      <c r="B27" s="6" t="inlineStr">
-        <is>
-          <t>accede</t>
-        </is>
-      </c>
-      <c r="C27" s="6" t="inlineStr">
-        <is>
-          <t>animate</t>
-        </is>
-      </c>
-      <c r="D27" s="6" t="inlineStr">
-        <is>
-          <t>curtail</t>
-        </is>
-      </c>
-      <c r="E27" s="6" t="inlineStr">
-        <is>
-          <t>abstain</t>
-        </is>
-      </c>
-      <c r="F27" s="7" t="n">
-        <v>20</v>
-      </c>
-      <c r="G27" s="7" t="n">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="28" ht="30" customHeight="1">
-      <c r="A28" s="6" t="inlineStr">
-        <is>
-          <t>Which word means "showing care in doing one's work"?</t>
-        </is>
-      </c>
-      <c r="B28" s="6" t="inlineStr">
-        <is>
-          <t>diligent</t>
-        </is>
-      </c>
-      <c r="C28" s="6" t="inlineStr">
-        <is>
-          <t>boisterous</t>
-        </is>
-      </c>
-      <c r="D28" s="6" t="inlineStr">
-        <is>
-          <t>cunning</t>
-        </is>
-      </c>
-      <c r="E28" s="6" t="inlineStr">
-        <is>
-          <t>affluent</t>
-        </is>
-      </c>
-      <c r="F28" s="7" t="n">
-        <v>20</v>
-      </c>
-      <c r="G28" s="7" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="8" t="inlineStr">
-        <is>
-          <t>Rows 9-18 ask term to definition; the shaded rows 19-28 ask definition to term. Blue text = the text Kahoot shows players. Words and definitions transcribed from the LINCS worksheets; part of speech, synonyms, sentences and pictures were left out on request.</t>
+          <t>Rows 9-18 each show a word and ask for its meaning. Blue text = the text Kahoot shows players. Words and definitions transcribed from the LINCS worksheets; part of speech, synonyms, sentences and pictures were left out on request.</t>
         </is>
       </c>
     </row>

</xml_diff>